<commit_message>
Update test results printour
</commit_message>
<xml_diff>
--- a/Fortran/results/Test_results.xlsx
+++ b/Fortran/results/Test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\proek\Documents\GitHub\ModAB-Root-Finding\Fortran\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DB781E-9DC0-49C1-A017-5BB2927719AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBB1433-71F2-4E6B-A7A1-B360BF188051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{901E7075-F730-4135-A5B3-71A5C4E5AAAF}"/>
   </bookViews>
@@ -2396,7 +2396,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BO237"/>
+  <dimension ref="A1:BO236"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.26953125" customWidth="1"/>
@@ -57089,7 +57089,9 @@
       </c>
     </row>
     <row r="227" spans="1:67" x14ac:dyDescent="0.35">
-      <c r="A227" s="11"/>
+      <c r="A227" s="11" t="s">
+        <v>214</v>
+      </c>
       <c r="B227" s="11"/>
       <c r="C227" s="11"/>
       <c r="D227" s="11"/>
@@ -58455,77 +58457,6 @@
       <c r="BN236" s="11"/>
       <c r="BO236" s="11"/>
     </row>
-    <row r="237" spans="1:67" x14ac:dyDescent="0.35">
-      <c r="A237" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="B237" s="11"/>
-      <c r="C237" s="11"/>
-      <c r="D237" s="11"/>
-      <c r="E237" s="11"/>
-      <c r="F237" s="11"/>
-      <c r="G237" s="11"/>
-      <c r="H237" s="11"/>
-      <c r="I237" s="11"/>
-      <c r="J237" s="11"/>
-      <c r="K237" s="11"/>
-      <c r="L237" s="11"/>
-      <c r="M237" s="11"/>
-      <c r="N237" s="11"/>
-      <c r="O237" s="11"/>
-      <c r="P237" s="11"/>
-      <c r="Q237" s="11"/>
-      <c r="R237" s="11"/>
-      <c r="S237" s="11"/>
-      <c r="T237" s="11"/>
-      <c r="U237" s="11"/>
-      <c r="V237" s="11"/>
-      <c r="W237" s="11"/>
-      <c r="X237" s="11"/>
-      <c r="Y237" s="11"/>
-      <c r="Z237" s="11"/>
-      <c r="AA237" s="11"/>
-      <c r="AB237" s="11"/>
-      <c r="AC237" s="11"/>
-      <c r="AD237" s="11"/>
-      <c r="AE237" s="11"/>
-      <c r="AF237" s="11"/>
-      <c r="AG237" s="11"/>
-      <c r="AH237" s="11"/>
-      <c r="AI237" s="11"/>
-      <c r="AJ237" s="11"/>
-      <c r="AK237" s="11"/>
-      <c r="AL237" s="11"/>
-      <c r="AM237" s="11"/>
-      <c r="AN237" s="11"/>
-      <c r="AO237" s="11"/>
-      <c r="AP237" s="11"/>
-      <c r="AQ237" s="11"/>
-      <c r="AR237" s="11"/>
-      <c r="AS237" s="11"/>
-      <c r="AT237" s="11"/>
-      <c r="AU237" s="11"/>
-      <c r="AV237" s="11"/>
-      <c r="AW237" s="11"/>
-      <c r="AX237" s="11"/>
-      <c r="AY237" s="11"/>
-      <c r="AZ237" s="11"/>
-      <c r="BA237" s="11"/>
-      <c r="BB237" s="11"/>
-      <c r="BC237" s="11"/>
-      <c r="BD237" s="11"/>
-      <c r="BE237" s="11"/>
-      <c r="BF237" s="11"/>
-      <c r="BG237" s="11"/>
-      <c r="BH237" s="11"/>
-      <c r="BI237" s="11"/>
-      <c r="BJ237" s="11"/>
-      <c r="BK237" s="11"/>
-      <c r="BL237" s="11"/>
-      <c r="BM237" s="11"/>
-      <c r="BN237" s="11"/>
-      <c r="BO237" s="11"/>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="F3:Y225">
     <cfRule type="colorScale" priority="4">
@@ -58559,8 +58490,8 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.55118110236220474" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="22" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="41" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>